<commit_message>
Split NSN Cosmetics summary into 3 HS codes after TARIC review
Reclassified from shipper's blanket 3304.30: scrubs/gels/lotions to
3304990000 (0%), Spa Salt to 3307300000 (6.5%), liquid soap sample to
3401300000 (4%). Gross weight distributed proportionally to net.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018YWkaCWSKYi1eJRixEWy9n
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_NSN_Cosmetics_OOCU9479533.xlsx
+++ b/output/HS_Code_Summary_NSN_Cosmetics_OOCU9479533.xlsx
@@ -33,13 +33,13 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00C00000"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -49,6 +49,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE0B2"/>
       </patternFill>
     </fill>
   </fills>
@@ -78,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -88,13 +93,18 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -466,18 +476,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="55" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -527,15 +537,15 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="60" customHeight="1">
+    <row r="2" ht="55" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>3304300000</t>
+          <t>3304990000</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Kosmetické přípravky pro manikúru a pedikúru – peeling na nohy (Sugar Scrub), sůl do koupele (Spa Salt), masážní gel na nohy s mátou (Gel Scrub Mint), krémy na nohy (Lotion), tekuté mýdlo na ruce (Lotion Soap)</t>
+          <t>Ostatní kosmetické přípravky pro péči o pokožku – peeling na nohy (Sugar Scrub), masážní gel na nohy s mátou (Gel Scrub Mint), krémy na nohy (Lotion)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -544,106 +554,168 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
+        <v>755</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>14306.3</v>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>14289.77</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>19168.86</v>
+      </c>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Smluvní clo třetí země 0 %. Přeřazeno z deklarovaného 3304.30 (manikúra/pedikúra) – jde o péči o pokožku, ne o nehty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="55" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>3307300000</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Vonné soli a jiné přípravky do koupele – sůl do koupele Spa Salt, modrá (balení 5 gal a 1 gal)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>259</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>5647.23</v>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>5640.7</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>4625.82</v>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>CLO 6,5 %</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>Smluvní clo třetí země 6,5 % (≈ 300 USD). Přeřazeno z deklarovaného 3304.30 – soli do koupele jsou jmenovitě uvedeny v 3307 30. Bez preference (USA).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="55" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>3401300000</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Organické povrchově aktivní prostředky k mytí pokožky, tekuté – tekuté mýdlo na ruce (vzorek, 1 ks)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>4.54</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>4.53</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>5.32</v>
+      </c>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Smluvní clo třetí země 4 % (hodnota 5,32 USD – zanedbatelné). Přeřazeno z deklarovaného 3304.30.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="55" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>CELKEM</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="n"/>
+      <c r="C5" s="9" t="n"/>
+      <c r="D5" s="9" t="n">
         <v>1015</v>
       </c>
-      <c r="E2" s="4" t="n">
-        <v>19958.06</v>
-      </c>
-      <c r="F2" s="4" t="n">
+      <c r="E5" s="11" t="n">
+        <v>19958.07</v>
+      </c>
+      <c r="F5" s="11" t="n">
         <v>19935</v>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="G5" s="11" t="n">
         <v>23800</v>
       </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>POZOR</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Bez preferenční věty (USA – žádná preference s EU neexistuje, platí sazba třetí země; dle TARIC pro 3304 30 00 je smluvní clo 0 % – ověřit při podání). Nesoulad hmotností a kusů – viz legenda a list Poznámky.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>CELKEM</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="n"/>
-      <c r="C3" s="6" t="n"/>
-      <c r="D3" s="6" t="n">
-        <v>1015</v>
-      </c>
-      <c r="E3" s="8" t="n">
-        <v>19958.06</v>
-      </c>
-      <c r="F3" s="8" t="n">
-        <v>19935</v>
-      </c>
-      <c r="G3" s="8" t="n">
-        <v>23800</v>
-      </c>
-      <c r="H3" s="6" t="n"/>
-      <c r="I3" s="6" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="H5" s="9" t="n"/>
+      <c r="I5" s="10" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Legenda:</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>⚠️ PREFERENČNÍ VĚTA: v žádném z 5 dokumentů (obchodní faktura 952626, HBL, MBL, D/O, freight faktura) NENÍ preferenční věta. Původ USA – EU nemá s USA preferenční dohodu, uplatní se standardní sazba třetí země.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>⚠️ HMOTNOSTI: faktura uvádí NET 44 000 lbs (= 19 958,06 kg) a sloupec „Gross (KGS)“ 19 958 kg – to je jen přepočet téhož čísla lbs→kg, nikoli skutečná hrubá hmotnost. B/L uvádí gross 19 935 kg. Skutečná čistá hmotnost není v dokladech samostatně uvedena – vyžádat od shippera.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="B8" s="10" t="inlineStr">
+    <row r="8" ht="42" customHeight="1">
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>⚠️ PREFERENČNÍ VĚTA: v žádném z 5 dokumentů NENÍ preferenční věta. Původ USA – EU nemá s USA preferenční dohodu, uplatní se standardní sazba třetí země (3304 99: 0 %, 3307 30: 6,5 %, 3401 30: 4 %). DPH 21 %.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1">
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>⚠️ PŘEŘAZENÍ HS: shipper deklaroval vše pod 3304.30.00.00 (manikúra/pedikúra). Dle TARIC jde o jiné zboží – rozděleno na 3 kódy (viz sloupec poznámka). US export kód není pro dovoz do EU závazný.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>⚠️ HMOTNOSTI: faktura uvádí NET 44 000 lbs (= 19 958,06 kg); sloupec „Gross (KGS)“ na faktuře je jen přepočet lbs→kg, nikoli skutečná GW. B/L gross 19 935 kg &lt; přepočtená NET → skutečná čistá hmotnost chybí, vyžádat od shippera. GW rozdělena proporcionálně dle NET (faktor 0,99885).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>⚠️ POČET KUSŮ: faktura = 1 015 ks, HBL/MBL/D/O = 1 032 ks. Rozdíl 17 ks – vyjasnit před podáním JSD.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>CBAM: NE – kosmetika nespadá do působnosti CBAM.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>ANTIDUMPING: NE – na HS 3304 30 00 z USA se antidumpingové clo nevztahuje.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>SLEVA: žádná obchodní sleva na faktuře – hodnota bez úprav.</t>
+    <row r="12" ht="42" customHeight="1">
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>CBAM: NE – kosmetika/mýdlo nespadá do působnosti CBAM. ANTIDUMPING: NE (původ USA). SLEVA: žádná.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="5">
     <mergeCell ref="B9:I9"/>
-    <mergeCell ref="B7:I7"/>
+    <mergeCell ref="B12:I12"/>
     <mergeCell ref="B11:I11"/>
-    <mergeCell ref="B6:I6"/>
     <mergeCell ref="B10:I10"/>
     <mergeCell ref="B8:I8"/>
   </mergeCells>
@@ -657,62 +729,68 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="6" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="14" t="inlineStr">
         <is>
           <t>Položka (faktura)</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="14" t="inlineStr">
         <is>
           <t>Český popis (z instrukcí)</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
-        <is>
-          <t>HS kód (deklarovaný)</t>
-        </is>
-      </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="D1" s="14" t="inlineStr">
+        <is>
+          <t>HS kód (JSD)</t>
+        </is>
+      </c>
+      <c r="E1" s="14" t="inlineStr">
+        <is>
+          <t>HS deklarovaný shipperem</t>
+        </is>
+      </c>
+      <c r="F1" s="14" t="inlineStr">
         <is>
           <t>Ks</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="G1" s="14" t="inlineStr">
         <is>
           <t>Net (lbs)</t>
         </is>
       </c>
-      <c r="G1" s="11" t="inlineStr">
+      <c r="H1" s="14" t="inlineStr">
         <is>
           <t>Hmotnost (kg)*</t>
         </is>
       </c>
-      <c r="H1" s="11" t="inlineStr">
+      <c r="I1" s="14" t="inlineStr">
         <is>
           <t>Cena USD</t>
         </is>
       </c>
-      <c r="I1" s="11" t="inlineStr">
+      <c r="J1" s="14" t="inlineStr">
         <is>
           <t>COO</t>
         </is>
@@ -734,22 +812,27 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>3304990000</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>3304.30.00.00</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="F2" s="2" t="n">
         <v>288</v>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="G2" s="2" t="n">
         <v>15360</v>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="H2" s="2" t="n">
         <v>6967</v>
       </c>
-      <c r="H2" s="4" t="n">
+      <c r="I2" s="4" t="n">
         <v>11520</v>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>US</t>
         </is>
@@ -771,22 +854,27 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>3307300000</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
           <t>3304.30.00.00</t>
         </is>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="F3" s="2" t="n">
         <v>192</v>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="G3" s="2" t="n">
         <v>9440</v>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="H3" s="2" t="n">
         <v>4282</v>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="I3" s="4" t="n">
         <v>3456</v>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>US</t>
         </is>
@@ -808,22 +896,27 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
+          <t>3307300000</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
           <t>3304.30.00.00</t>
         </is>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="F4" s="2" t="n">
         <v>67</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="G4" s="2" t="n">
         <v>3010</v>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="H4" s="2" t="n">
         <v>1365</v>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="I4" s="4" t="n">
         <v>1169.82</v>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>US</t>
         </is>
@@ -845,22 +938,27 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
+          <t>3304990000</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
           <t>3304.30.00.00</t>
         </is>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="F5" s="2" t="n">
         <v>96</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="G5" s="2" t="n">
         <v>4060</v>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="H5" s="2" t="n">
         <v>1842</v>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="I5" s="4" t="n">
         <v>1728</v>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>US</t>
         </is>
@@ -882,22 +980,27 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
+          <t>3304990000</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
           <t>3304.30.00.00</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="F6" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="G6" s="2" t="n">
         <v>2220</v>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="H6" s="2" t="n">
         <v>1007</v>
       </c>
-      <c r="H6" s="4" t="n">
+      <c r="I6" s="4" t="n">
         <v>960</v>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>US</t>
         </is>
@@ -919,22 +1022,27 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
+          <t>3304990000</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
           <t>3304.30.00.00</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="F7" s="2" t="n">
         <v>141</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="G7" s="2" t="n">
         <v>4540</v>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="H7" s="2" t="n">
         <v>2059</v>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="I7" s="4" t="n">
         <v>2109.36</v>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>US</t>
         </is>
@@ -956,22 +1064,27 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
+          <t>3304990000</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
           <t>3304.30.00.00</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="F8" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="G8" s="2" t="n">
         <v>740</v>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="H8" s="2" t="n">
         <v>336</v>
       </c>
-      <c r="H8" s="4" t="n">
+      <c r="I8" s="4" t="n">
         <v>720</v>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>US</t>
         </is>
@@ -993,22 +1106,27 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
+          <t>3304990000</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
           <t>3304.30.00.00</t>
         </is>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="F9" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="G9" s="2" t="n">
         <v>3720</v>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="H9" s="2" t="n">
         <v>1687</v>
       </c>
-      <c r="H9" s="4" t="n">
+      <c r="I9" s="4" t="n">
         <v>1740</v>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>US</t>
         </is>
@@ -1030,22 +1148,27 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
+          <t>3304990000</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
           <t>3304.30.00.00</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="F10" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="G10" s="2" t="n">
         <v>900</v>
       </c>
-      <c r="G10" s="2" t="n">
+      <c r="H10" s="2" t="n">
         <v>408</v>
       </c>
-      <c r="H10" s="4" t="n">
+      <c r="I10" s="4" t="n">
         <v>391.5</v>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>US</t>
         </is>
@@ -1067,49 +1190,55 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
+          <t>3401300000</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
           <t>3304.30.00.00</t>
         </is>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="F11" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="2" t="n">
+      <c r="G11" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="G11" s="2" t="n">
+      <c r="H11" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H11" s="4" t="n">
+      <c r="I11" s="4" t="n">
         <v>5.32</v>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr"/>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr"/>
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>CELKEM</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="6" t="n">
+      <c r="C12" s="10" t="n"/>
+      <c r="D12" s="9" t="n"/>
+      <c r="E12" s="9" t="n"/>
+      <c r="F12" s="9" t="n">
         <v>1015</v>
       </c>
-      <c r="F12" s="6" t="n">
+      <c r="G12" s="9" t="n">
         <v>44000</v>
       </c>
-      <c r="G12" s="6" t="n">
+      <c r="H12" s="9" t="n">
         <v>19958</v>
       </c>
-      <c r="H12" s="8" t="n">
+      <c r="I12" s="11" t="n">
         <v>23800</v>
       </c>
-      <c r="I12" s="6" t="n"/>
+      <c r="J12" s="9" t="n"/>
     </row>
     <row r="14">
       <c r="B14" t="inlineStr">
@@ -1129,14 +1258,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A40"/>
+  <dimension ref="A1:A45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9">
+      <c r="A1" s="12">
         <f>== ZÁSILKA ===</f>
         <v/>
       </c>
@@ -1201,7 +1330,7 @@
       <c r="A10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="9">
+      <c r="A11" s="12">
         <f>== PŘIJATÉ DOKUMENTY (stav 13.7.2026) ===</f>
         <v/>
       </c>
@@ -1209,7 +1338,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>✓ Obchodní faktura / packing list Cali Chem č. 952626 z 29.5.2026 – 10 položek, 23 800,00 USD, vše HS 3304.30.00.00, COO USA</t>
+          <t>✓ Obchodní faktura / packing list Cali Chem č. 952626 z 29.5.2026 – 10 položek, 23 800,00 USD, COO USA</t>
         </is>
       </c>
     </row>
@@ -1252,138 +1381,168 @@
       <c r="A18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="9">
+      <c r="A19" s="12">
+        <f>== SAZEBNÍ ZAŘAZENÍ – ROZHODNUTÍ (13.7.2026) ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Shipper deklaroval všech 10 položek pod 3304.30.00.00 (přípravky pro manikúru nebo pedikúru).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Po kontrole TARIC rozděleno na 3 kódy (US export kód není pro dovoz do EU závazný):</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • 3304 99 00 00 – peelingy, gely, krémy na nohy (péče o pokožku, ne o nehty) … clo 0 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • 3307 30 00 00 – Spa Salt = sůl do koupele, jmenovitě uvedena v 3307 30 … clo 6,5 % (≈ 300 USD z 4 625,82 USD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • 3401 30 00 00 – tekuté mýdlo na ruce, vzorek 1 ks … clo 4 % (z 5,32 USD, zanedbatelné)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Sazby ověřit v TARIC při podání JSD. U soli by definitivu dalo složení / product datasheet, příp. ZISZ (BTI).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="12">
         <f>== ⚠️ PREFERENČNÍ VĚTA – NENÍ ===</f>
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>Žádný dokument neobsahuje preferenční větu (prohlášení o preferenčním původu).</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>Původ zboží: USA. EU nemá s USA preferenční obchodní dohodu → preferenci nelze uplatnit a věta se ani nevyžaduje.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Platí smluvní sazba třetí země; dle TARIC je u 3304 30 00 00 smluvní clo 0 % (ověřit při podání JSD). DPH 21 %.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="9">
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Platí smluvní sazby třetí země (viz výše). DPH 21 %.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="12">
         <f>== ⚠️ NESROVNALOSTI K VYJASNĚNÍ ===</f>
         <v/>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>1) POČET KUSŮ: faktura 1 015 ks vs. HBL/MBL/D/O 1 032 ks (SLAC). Rozdíl 17 ks – vyjasnit se shipperem/forwarderem.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>2) HMOTNOSTI: faktura Net 44 000 lbs = 19 958,06 kg; sloupec Gross (KGS) 19 958 kg je jen přepočet lbs→kg (není to skutečná GW).</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   B/L gross 19 935 kg &lt; „net“ 19 958 kg → fyzicky nemožné. Skutečná NET hmotnost chybí – vyžádat od shippera.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Pro JSD zatím: GW 19 935 kg (dle B/L); NW nutno doložit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>3) SAZEBNÍ ZAŘAZENÍ: vše deklarováno pod 3304.30 (přípravky pro manikúru/pedikúru). Pozor – „sůl do koupele“ obvykle patří</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   do 3307 30 00 a „tekuté mýdlo na ruce“ do 3401 30 00. Vzhledem k určení (pedikúra/nail salon) je 3304.30 obhajitelné,</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   ale doporučuji potvrdit zařazení položek 2, 3 a 10 před podáním.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>4) INCOTERM: na faktuře není uveden; B/L „Freight Prepaid“. Ocean freight 3 700 USD hradí shipper → pro celní hodnotu</t>
-        </is>
-      </c>
-    </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>1) POČET KUSŮ: faktura 1 015 ks vs. HBL/MBL/D/O 1 032 ks (SLAC). Rozdíl 17 ks – vyjasnit se shipperem/forwarderem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2) HMOTNOSTI: faktura Net 44 000 lbs = 19 958,06 kg; sloupec Gross (KGS) 19 958 kg je jen přepočet lbs→kg (není to skutečná GW).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   B/L gross 19 935 kg &lt; „net“ 19 958 kg → fyzicky nemožné. Skutečná NET hmotnost chybí – vyžádat od shippera.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Pro JSD zatím: GW 19 935 kg (dle B/L), rozdělena proporcionálně dle NET; NW nutno doložit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>3) INCOTERM: na faktuře není uveden; B/L „Freight Prepaid“. Ocean freight 3 700 USD hradí shipper → pro celní hodnotu</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t xml:space="preserve">   ověřit dodací podmínku (při CFR/CIF je přeprava již v ceně; při FOB/EXW nutno přičíst přepravu k celní hodnotě).</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="9">
+    <row r="39">
+      <c r="A39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="12">
         <f>== CBAM / ANTIDUMPING ===</f>
         <v/>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>CBAM: nevztahuje se (kosmetické přípravky).</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Antidumping: nevztahuje se (HS 3304 30 00, původ USA).</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="9">
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>CBAM: nevztahuje se (kosmetické přípravky, mýdlo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Antidumping: nevztahuje se (kap. 33/34, původ USA).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="12">
         <f>== SLEVA ===</f>
         <v/>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
+    <row r="45">
+      <c r="A45" t="inlineStr">
         <is>
           <t>Žádná obchodní sleva na faktuře – celní hodnota bez úprav: 23 800,00 USD.</t>
         </is>

</xml_diff>

<commit_message>
Apply tariff department ruling: massage gel to 3307900000
Per Marketa Navratilova's e-mail (13.7.2026): Gel Scrub Mint's main
purpose is massage, moisturizing is only secondary, so it moves from
3304990000 to 3307900000 (6.5% duty). Other codes confirmed. Added
chapter 33 retail-packaging condition warning to notes. Updated both
the HS summary and the instruction sheet.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018YWkaCWSKYi1eJRixEWy9n
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_NSN_Cosmetics_OOCU9479533.xlsx
+++ b/output/HS_Code_Summary_NSN_Cosmetics_OOCU9479533.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -545,7 +545,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Ostatní kosmetické přípravky pro péči o pokožku – peeling na nohy (Sugar Scrub), masážní gel na nohy s mátou (Gel Scrub Mint), krémy na nohy (Lotion)</t>
+          <t>Ostatní kosmetické přípravky pro péči o pokožku – peeling na nohy (Sugar Scrub), krémy na nohy (Lotion)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -554,21 +554,21 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>755</v>
+        <v>599</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>14306.3</v>
+        <v>11457.74</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>14289.77</v>
+        <v>11444.5</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>19168.86</v>
+        <v>16480.86</v>
       </c>
       <c r="H2" s="2" t="n"/>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Smluvní clo třetí země 0 %. Přeřazeno z deklarovaného 3304.30 (manikúra/pedikúra) – jde o péči o pokožku, ne o nehty.</t>
+          <t>Smluvní clo třetí země 0 %. Přeřazeno z deklarovaného 3304.30 (manikúra/pedikúra) – jde o péči o pokožku, ne o nehty. Potvrzeno TARIC odd. (M. Navrátilová, 13.7.2026).</t>
         </is>
       </c>
     </row>
@@ -607,117 +607,164 @@
       </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>Smluvní clo třetí země 6,5 % (≈ 300 USD). Přeřazeno z deklarovaného 3304.30 – soli do koupele jsou jmenovitě uvedeny v 3307 30. Bez preference (USA).</t>
+          <t>Smluvní clo třetí země 6,5 % (≈ 300,68 USD). Soli do koupele jmenovitě v 3307 30. Potvrzeno TARIC odd. (M. Navrátilová). Bez preference (USA).</t>
         </is>
       </c>
     </row>
     <row r="4" ht="55" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>3307900000</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Ostatní voňavkářské, kosmetické nebo toaletní přípravky – aromaterapeutický masážní gel na nohy s mátou (Gel Scrub Mint)</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>156</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>2848.56</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>2845.27</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>2688</v>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>CLO 6,5 %</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Smluvní clo třetí země 6,5 % (≈ 174,72 USD). Dle stanoviska TARIC odd. (M. Navrátilová, 13.7.2026): hlavním určením je masáž, hydratační účinek jen doprovodný → 3307 90, nikoli 3304.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="55" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>3401300000</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Organické povrchově aktivní prostředky k mytí pokožky, tekuté – tekuté mýdlo na ruce (vzorek, 1 ks)</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E5" s="4" t="n">
         <v>4.54</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="F5" s="4" t="n">
         <v>4.53</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="G5" s="4" t="n">
         <v>5.32</v>
       </c>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Smluvní clo třetí země 4 % (hodnota 5,32 USD – zanedbatelné). Přeřazeno z deklarovaného 3304.30.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="55" customHeight="1">
-      <c r="A5" s="9" t="inlineStr">
+    <row r="6" ht="55" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>CELKEM</t>
         </is>
       </c>
-      <c r="B5" s="10" t="n"/>
-      <c r="C5" s="9" t="n"/>
-      <c r="D5" s="9" t="n">
+      <c r="B6" s="10" t="n"/>
+      <c r="C6" s="9" t="n"/>
+      <c r="D6" s="9" t="n">
         <v>1015</v>
       </c>
-      <c r="E5" s="11" t="n">
+      <c r="E6" s="11" t="n">
         <v>19958.07</v>
       </c>
-      <c r="F5" s="11" t="n">
+      <c r="F6" s="11" t="n">
         <v>19935</v>
       </c>
-      <c r="G5" s="11" t="n">
+      <c r="G6" s="11" t="n">
         <v>23800</v>
       </c>
-      <c r="H5" s="9" t="n"/>
-      <c r="I5" s="10" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="H6" s="9" t="n"/>
+      <c r="I6" s="10" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Legenda:</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="42" customHeight="1">
-      <c r="B8" s="13" t="inlineStr">
-        <is>
-          <t>⚠️ PREFERENČNÍ VĚTA: v žádném z 5 dokumentů NENÍ preferenční věta. Původ USA – EU nemá s USA preferenční dohodu, uplatní se standardní sazba třetí země (3304 99: 0 %, 3307 30: 6,5 %, 3401 30: 4 %). DPH 21 %.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1">
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>⚠️ PŘEŘAZENÍ HS: shipper deklaroval vše pod 3304.30.00.00 (manikúra/pedikúra). Dle TARIC jde o jiné zboží – rozděleno na 3 kódy (viz sloupec poznámka). US export kód není pro dovoz do EU závazný.</t>
+          <t>⚠️ PREFERENČNÍ VĚTA: v žádném z 5 dokumentů NENÍ preferenční věta. Původ USA – EU nemá s USA preferenční dohodu, uplatní se standardní sazba třetí země (3304 99: 0 %, 3307 30 a 3307 90: 6,5 %, 3401 30: 4 %). DPH 21 %. Odhad cla celkem ≈ 475,61 USD.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1">
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>⚠️ HMOTNOSTI: faktura uvádí NET 44 000 lbs (= 19 958,06 kg); sloupec „Gross (KGS)“ na faktuře je jen přepočet lbs→kg, nikoli skutečná GW. B/L gross 19 935 kg &lt; přepočtená NET → skutečná čistá hmotnost chybí, vyžádat od shippera. GW rozdělena proporcionálně dle NET (faktor 0,99885).</t>
+          <t>⚠️ PŘEŘAZENÍ HS: shipper deklaroval vše pod 3304.30.00.00 (manikúra/pedikúra). Jednotné zařazení není možné (rozdílný objektivní charakter a způsob použití) – rozděleno na 4 kódy dle stanoviska TARIC oddělení (M. Navrátilová, e-mail 13.7.2026). US export kód není pro dovoz do EU závazný.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1">
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>⚠️ POČET KUSŮ: faktura = 1 015 ks, HBL/MBL/D/O = 1 032 ks. Rozdíl 17 ks – vyjasnit před podáním JSD.</t>
+          <t>⚠️ PODMÍNKA KAP. 33 (upozornění TARIC odd.): u výrobků čísel 3304 a 3307 musí být splněna podmínka pozn. 3 ke kap. 33 – přípravky „v odměřených dávkách nebo upravené ve formě či balení pro drobný prodej“. Zboží je v salonních baleních 1–5 gal (20 kg) – ověřit s TARIC odd., že balení podmínku splňuje.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="B12" s="13" t="inlineStr">
         <is>
+          <t>⚠️ HMOTNOSTI: faktura uvádí NET 44 000 lbs (= 19 958,06 kg); sloupec „Gross (KGS)“ na faktuře je jen přepočet lbs→kg, nikoli skutečná GW. B/L gross 19 935 kg &lt; přepočtená NET → skutečná čistá hmotnost chybí, vyžádat od shippera. GW rozdělena proporcionálně dle NET (faktor 0,99885).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>⚠️ POČET KUSŮ: faktura = 1 015 ks, HBL/MBL/D/O = 1 032 ks. Rozdíl 17 ks – vyjasnit před podáním JSD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1">
+      <c r="B14" s="13" t="inlineStr">
+        <is>
           <t>CBAM: NE – kosmetika/mýdlo nespadá do působnosti CBAM. ANTIDUMPING: NE (původ USA). SLEVA: žádná.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="B9:I9"/>
+    <mergeCell ref="B13:I13"/>
     <mergeCell ref="B12:I12"/>
     <mergeCell ref="B11:I11"/>
     <mergeCell ref="B10:I10"/>
-    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="B14:I14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -938,7 +985,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>3304990000</t>
+          <t>3307900000</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -980,7 +1027,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>3304990000</t>
+          <t>3307900000</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -1258,7 +1305,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A45"/>
+  <dimension ref="A1:A50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -1382,7 +1429,7 @@
     </row>
     <row r="19">
       <c r="A19" s="12">
-        <f>== SAZEBNÍ ZAŘAZENÍ – ROZHODNUTÍ (13.7.2026) ===</f>
+        <f>== SAZEBNÍ ZAŘAZENÍ – POTVRZENO TARIC ODDĚLENÍM (M. Navrátilová, e-mail 13.7.2026) ===</f>
         <v/>
       </c>
     </row>
@@ -1396,153 +1443,188 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Po kontrole TARIC rozděleno na 3 kódy (US export kód není pro dovoz do EU závazný):</t>
+          <t>Stanovisko TARIC odd.: jednotné zařazení do 3304 30 NENÍ možné – výrobky mají rozdílný objektivní charakter a způsob použití.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • 3304 99 00 00 – peelingy, gely, krémy na nohy (péče o pokožku, ne o nehty) … clo 0 %</t>
+          <t>Konečné rozdělení na 4 kódy:</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • 3307 30 00 00 – Spa Salt = sůl do koupele, jmenovitě uvedena v 3307 30 … clo 6,5 % (≈ 300 USD z 4 625,82 USD)</t>
+          <t xml:space="preserve">  • 3304 99 00 00 – peeling na nohy (Sugar Scrub), krémy na nohy (Lotion) … clo 0 %</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • 3401 30 00 00 – tekuté mýdlo na ruce, vzorek 1 ks … clo 4 % (z 5,32 USD, zanedbatelné)</t>
+          <t xml:space="preserve">  • 3307 30 00 00 – Spa Salt = sůl do koupele … clo 6,5 % (≈ 300,68 USD z 4 625,82 USD)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Sazby ověřit v TARIC při podání JSD. U soli by definitivu dalo složení / product datasheet, příp. ZISZ (BTI).</t>
+          <t xml:space="preserve">  • 3307 90 00 00 – Gel Scrub Mint = masážní gel na nohy … clo 6,5 % (≈ 174,72 USD z 2 688,00 USD)</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr"/>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    (dle TARIC odd.: hlavním určením je masáž, hydratační účinek pouze doprovodný → nelze do 3304)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="12">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • 3401 30 00 00 – tekuté mýdlo na ruce, vzorek 1 ks … clo 4 % (z 5,32 USD, zanedbatelné)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>⚠️ Upozornění TARIC odd.: u čísel 3304 a 3307 musí být splněna podmínka pozn. ke kap. 33 – přípravky</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>„v odměřených dávkách nebo upravené ve formě či balení pro drobný prodej“. Balení je salonní (1–5 gal / 20 kg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>– ověřit, že splňuje; jinak hrozí přeřazení mimo kap. 33.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="12">
         <f>== ⚠️ PREFERENČNÍ VĚTA – NENÍ ===</f>
         <v/>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>Žádný dokument neobsahuje preferenční větu (prohlášení o preferenčním původu).</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+    <row r="34">
+      <c r="A34" t="inlineStr">
         <is>
           <t>Původ zboží: USA. EU nemá s USA preferenční obchodní dohodu → preferenci nelze uplatnit a věta se ani nevyžaduje.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t>Platí smluvní sazby třetí země (viz výše). DPH 21 %.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="12">
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="12">
         <f>== ⚠️ NESROVNALOSTI K VYJASNĚNÍ ===</f>
         <v/>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>1) POČET KUSŮ: faktura 1 015 ks vs. HBL/MBL/D/O 1 032 ks (SLAC). Rozdíl 17 ks – vyjasnit se shipperem/forwarderem.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>2) HMOTNOSTI: faktura Net 44 000 lbs = 19 958,06 kg; sloupec Gross (KGS) 19 958 kg je jen přepočet lbs→kg (není to skutečná GW).</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   B/L gross 19 935 kg &lt; „net“ 19 958 kg → fyzicky nemožné. Skutečná NET hmotnost chybí – vyžádat od shippera.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Pro JSD zatím: GW 19 935 kg (dle B/L), rozdělena proporcionálně dle NET; NW nutno doložit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>3) INCOTERM: na faktuře není uveden; B/L „Freight Prepaid“. Ocean freight 3 700 USD hradí shipper → pro celní hodnotu</t>
-        </is>
-      </c>
-    </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>1) POČET KUSŮ: faktura 1 015 ks vs. HBL/MBL/D/O 1 032 ks (SLAC). Rozdíl 17 ks – vyjasnit se shipperem/forwarderem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2) HMOTNOSTI: faktura Net 44 000 lbs = 19 958,06 kg; sloupec Gross (KGS) 19 958 kg je jen přepočet lbs→kg (není to skutečná GW).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   B/L gross 19 935 kg &lt; „net“ 19 958 kg → fyzicky nemožné. Skutečná NET hmotnost chybí – vyžádat od shippera.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Pro JSD zatím: GW 19 935 kg (dle B/L), rozdělena proporcionálně dle NET; NW nutno doložit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>3) INCOTERM: na faktuře není uveden; B/L „Freight Prepaid“. Ocean freight 3 700 USD hradí shipper → pro celní hodnotu</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t xml:space="preserve">   ověřit dodací podmínku (při CFR/CIF je přeprava již v ceně; při FOB/EXW nutno přičíst přepravu k celní hodnotě).</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="12">
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="12">
         <f>== CBAM / ANTIDUMPING ===</f>
         <v/>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
+    <row r="46">
+      <c r="A46" t="inlineStr">
         <is>
           <t>CBAM: nevztahuje se (kosmetické přípravky, mýdlo).</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
+    <row r="47">
+      <c r="A47" t="inlineStr">
         <is>
           <t>Antidumping: nevztahuje se (kap. 33/34, původ USA).</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="12">
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="12">
         <f>== SLEVA ===</f>
         <v/>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
+    <row r="50">
+      <c r="A50" t="inlineStr">
         <is>
           <t>Žádná obchodní sleva na faktuře – celní hodnota bez úprav: 23 800,00 USD.</t>
         </is>

</xml_diff>

<commit_message>
Update NSN Cosmetics summary with revised CI/PL weights
Revised invoice 952626 v2 states net and gross both in kg (net
19,123 / gross 19,935, matching the B/L), replacing the lbs-conversion
figures. Weights are now real per-item invoice values instead of the
proportional gross estimate. Piece-count discrepancy (1,015 vs 1,032)
still open. Added customs value note: freight billed to consignee,
add USD 3,795 transport to the customs value.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018YWkaCWSKYi1eJRixEWy9n
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_NSN_Cosmetics_OOCU9479533.xlsx
+++ b/output/HS_Code_Summary_NSN_Cosmetics_OOCU9479533.xlsx
@@ -557,10 +557,10 @@
         <v>599</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>11457.74</v>
+        <v>10948</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>11444.5</v>
+        <v>11434</v>
       </c>
       <c r="G2" s="4" t="n">
         <v>16480.86</v>
@@ -592,10 +592,10 @@
         <v>259</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>5647.23</v>
+        <v>5478</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>5640.7</v>
+        <v>5647</v>
       </c>
       <c r="G3" s="7" t="n">
         <v>4625.82</v>
@@ -631,10 +631,10 @@
         <v>156</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>2848.56</v>
+        <v>2693</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>2845.27</v>
+        <v>2849</v>
       </c>
       <c r="G4" s="7" t="n">
         <v>2688</v>
@@ -670,10 +670,10 @@
         <v>1</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>4.54</v>
+        <v>4</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>4.53</v>
+        <v>5</v>
       </c>
       <c r="G5" s="4" t="n">
         <v>5.32</v>
@@ -697,7 +697,7 @@
         <v>1015</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>19958.07</v>
+        <v>19123</v>
       </c>
       <c r="F6" s="11" t="n">
         <v>19935</v>
@@ -718,7 +718,7 @@
     <row r="9" ht="42" customHeight="1">
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>⚠️ PREFERENČNÍ VĚTA: v žádném z 5 dokumentů NENÍ preferenční věta. Původ USA – EU nemá s USA preferenční dohodu, uplatní se standardní sazba třetí země (3304 99: 0 %, 3307 30 a 3307 90: 6,5 %, 3401 30: 4 %). DPH 21 %. Odhad cla celkem ≈ 475,61 USD.</t>
+          <t>⚠️ PREFERENČNÍ VĚTA: v žádném dokumentu NENÍ preferenční věta. Původ USA – EU nemá s USA preferenční dohodu, uplatní se standardní sazba třetí země (3304 99: 0 %, 3307 30 a 3307 90: 6,5 %, 3401 30: 4 %). DPH 21 %. Odhad cla celkem ≈ 475,61 USD (z fakturní hodnoty; celní hodnota se navýší o přepravu – viz Poznámky).</t>
         </is>
       </c>
     </row>
@@ -739,14 +739,14 @@
     <row r="12" ht="42" customHeight="1">
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>⚠️ HMOTNOSTI: faktura uvádí NET 44 000 lbs (= 19 958,06 kg); sloupec „Gross (KGS)“ na faktuře je jen přepočet lbs→kg, nikoli skutečná GW. B/L gross 19 935 kg &lt; přepočtená NET → skutečná čistá hmotnost chybí, vyžádat od shippera. GW rozdělena proporcionálně dle NET (faktor 0,99885).</t>
+          <t>✓ HMOTNOSTI VYŘEŠENY: revidovaný CI/PL (v2, přijat 17.7.2026) uvádí NET i GROSS v kg. NET 19 123 kg, GROSS 19 935 kg = přesně dle B/L. Hmotnosti v tabulce jsou skutečné fakturní hodnoty po položkách.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1">
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>⚠️ POČET KUSŮ: faktura = 1 015 ks, HBL/MBL/D/O = 1 032 ks. Rozdíl 17 ks – vyjasnit před podáním JSD.</t>
+          <t>⚠️ POČET KUSŮ: faktura = 1 015 ks, HBL/MBL/D/O = 1 032 ks. Rozdíl 17 ks trvá i v revidovaném CI/PL – vyjasnit před podáním JSD.</t>
         </is>
       </c>
     </row>
@@ -786,7 +786,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
   </cols>
@@ -824,12 +824,12 @@
       </c>
       <c r="G1" s="14" t="inlineStr">
         <is>
-          <t>Net (lbs)</t>
+          <t>Net (kg)</t>
         </is>
       </c>
       <c r="H1" s="14" t="inlineStr">
         <is>
-          <t>Hmotnost (kg)*</t>
+          <t>Gross (kg)</t>
         </is>
       </c>
       <c r="I1" s="14" t="inlineStr">
@@ -871,7 +871,7 @@
         <v>288</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>15360</v>
+        <v>6792</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>6967</v>
@@ -913,7 +913,7 @@
         <v>192</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>9440</v>
+        <v>4180</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>4282</v>
@@ -955,7 +955,7 @@
         <v>67</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>3010</v>
+        <v>1298</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>1365</v>
@@ -997,7 +997,7 @@
         <v>96</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>4060</v>
+        <v>1746</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>1842</v>
@@ -1039,7 +1039,7 @@
         <v>60</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>2220</v>
+        <v>947</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>1007</v>
@@ -1081,10 +1081,10 @@
         <v>141</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>4540</v>
+        <v>1895</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>2059</v>
+        <v>2036</v>
       </c>
       <c r="I7" s="4" t="n">
         <v>2109.36</v>
@@ -1123,7 +1123,7 @@
         <v>20</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>740</v>
+        <v>316</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>336</v>
@@ -1165,7 +1165,7 @@
         <v>120</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>3720</v>
+        <v>1567</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>1687</v>
@@ -1207,7 +1207,7 @@
         <v>30</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>900</v>
+        <v>378</v>
       </c>
       <c r="H10" s="2" t="n">
         <v>408</v>
@@ -1249,7 +1249,7 @@
         <v>1</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>5</v>
@@ -1277,10 +1277,10 @@
         <v>1015</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>44000</v>
+        <v>19123</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>19958</v>
+        <v>19935</v>
       </c>
       <c r="I12" s="11" t="n">
         <v>23800</v>
@@ -1290,7 +1290,7 @@
     <row r="14">
       <c r="B14" t="inlineStr">
         <is>
-          <t>* Sloupec „Hmotnost (kg)“ na faktuře je označen jako Gross (KGS), ale je to pouze přepočet Net (lbs) → kg (faktor 0,4536).</t>
+          <t>Hmotnosti dle revidovaného CI/PL č. 952626 (v2) – NET i GROSS v kg; GROSS souhlasí s B/L (19 935 kg).</t>
         </is>
       </c>
     </row>
@@ -1305,7 +1305,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A50"/>
+  <dimension ref="A1:A55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -1378,255 +1378,285 @@
     </row>
     <row r="11">
       <c r="A11" s="12">
-        <f>== PŘIJATÉ DOKUMENTY (stav 13.7.2026) ===</f>
+        <f>== PŘIJATÉ DOKUMENTY (stav 17.7.2026) ===</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>✓ Obchodní faktura / packing list Cali Chem č. 952626 z 29.5.2026 – 10 položek, 23 800,00 USD, COO USA</t>
+          <t>✓ Obchodní faktura / packing list Cali Chem č. 952626 z 29.5.2026 – REVIDOVANÁ VERZE (v2, přijata 17.7.2026):</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>✓ HBL EHAM-W26JUN504 (WIN CARGO USA, 3 originály, shipped on board 7.6.2026)</t>
+          <t xml:space="preserve">   NET i GROSS nově v kg (NET 19 123 kg / GROSS 19 935 kg = souhlasí s B/L). 10 položek, 23 800,00 USD, COO USA.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>✓ MBL LAXHAM6160504V (Vanguard Logistics, express release, non-negotiable copy)</t>
+          <t xml:space="preserve">   Původní verze uváděla NET v lbs a jako GROSS jen přepočet lbs→kg – nahrazeno.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>✓ Delivery Order OOCL OOLU2327917280 (vyst. 9.7.2026), ATB: ATB1505238807202648510001</t>
+          <t>✓ HBL EHAM-W26JUN504 (WIN CARGO USA, 3 originály, shipped on board 7.6.2026)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>✓ Freight faktura WIN CARGO USA EHAM-W26JUN504 z 11.6.2026: ocean freight 3 700 USD + ENS 95 USD + bank fee 30 USD = 3 825 USD</t>
+          <t>✓ MBL LAXHAM6160504V (Vanguard Logistics, express release, non-negotiable copy)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>✓ Delivery Order OOCL OOLU2327917280 (vyst. 9.7.2026), ATB: ATB1505238807202648510001</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>✓ Freight faktura WIN CARGO USA EHAM-W26JUN504 z 11.6.2026: ocean freight 3 700 USD + ENS 95 USD + bank fee 30 USD = 3 825 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>✓ Instrukce k celnímu odbavení (INSTRUKCE_usa1.xlsx) – české popisy položek, hodnota 23 800 USD, JSD</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="12">
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="12">
         <f>== SAZEBNÍ ZAŘAZENÍ – POTVRZENO TARIC ODDĚLENÍM (M. Navrátilová, e-mail 13.7.2026) ===</f>
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Shipper deklaroval všech 10 položek pod 3304.30.00.00 (přípravky pro manikúru nebo pedikúru).</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Stanovisko TARIC odd.: jednotné zařazení do 3304 30 NENÍ možné – výrobky mají rozdílný objektivní charakter a způsob použití.</t>
-        </is>
-      </c>
-    </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Konečné rozdělení na 4 kódy:</t>
+          <t>Shipper deklaroval všech 10 položek pod 3304.30.00.00 (přípravky pro manikúru nebo pedikúru).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • 3304 99 00 00 – peeling na nohy (Sugar Scrub), krémy na nohy (Lotion) … clo 0 %</t>
+          <t>Stanovisko TARIC odd.: jednotné zařazení do 3304 30 NENÍ možné – výrobky mají rozdílný objektivní charakter a způsob použití.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • 3307 30 00 00 – Spa Salt = sůl do koupele … clo 6,5 % (≈ 300,68 USD z 4 625,82 USD)</t>
+          <t>Konečné rozdělení na 4 kódy:</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • 3307 90 00 00 – Gel Scrub Mint = masážní gel na nohy … clo 6,5 % (≈ 174,72 USD z 2 688,00 USD)</t>
+          <t xml:space="preserve">  • 3304 99 00 00 – peeling na nohy (Sugar Scrub), krémy na nohy (Lotion) … clo 0 %</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">    (dle TARIC odd.: hlavním určením je masáž, hydratační účinek pouze doprovodný → nelze do 3304)</t>
+          <t xml:space="preserve">  • 3307 30 00 00 – Spa Salt = sůl do koupele … clo 6,5 % (≈ 300,68 USD z 4 625,82 USD)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • 3401 30 00 00 – tekuté mýdlo na ruce, vzorek 1 ks … clo 4 % (z 5,32 USD, zanedbatelné)</t>
+          <t xml:space="preserve">  • 3307 90 00 00 – Gel Scrub Mint = masážní gel na nohy … clo 6,5 % (≈ 174,72 USD z 2 688,00 USD)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>⚠️ Upozornění TARIC odd.: u čísel 3304 a 3307 musí být splněna podmínka pozn. ke kap. 33 – přípravky</t>
+          <t xml:space="preserve">    (dle TARIC odd.: hlavním určením je masáž, hydratační účinek pouze doprovodný → nelze do 3304)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>„v odměřených dávkách nebo upravené ve formě či balení pro drobný prodej“. Balení je salonní (1–5 gal / 20 kg)</t>
+          <t xml:space="preserve">  • 3401 30 00 00 – tekuté mýdlo na ruce, vzorek 1 ks … clo 4 % (z 5,32 USD, zanedbatelné)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>⚠️ Upozornění TARIC odd.: u čísel 3304 a 3307 musí být splněna podmínka pozn. ke kap. 33 – přípravky</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>„v odměřených dávkách nebo upravené ve formě či balení pro drobný prodej“. Balení je salonní (1–5 gal / 20 kg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>– ověřit, že splňuje; jinak hrozí přeřazení mimo kap. 33.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="12">
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="12">
+        <f>== CELNÍ HODNOTA / INCOTERM ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Incoterm na CI/PL neuveden; B/L „Freight Prepaid“, ALE freight fakturuje WIN CARGO přímo NSN (příjemci)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>→ přepravu nese kupující (FOB-typ) → k celní hodnotě přičíst dopravu na hranici EU:</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   23 800,00 (zboží) + 3 700,00 (ocean freight) + 95,00 (ENS) ≈ 27 595,00 USD celní hodnota.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Bank fee 30 USD se do celní hodnoty nezahrnuje. Clo pak vychází ≈ 500 USD (6,5 % z podílu soli a gelu).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Do základu DPH vstupuje i doprava do místa určení v EU.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="12">
         <f>== ⚠️ PREFERENČNÍ VĚTA – NENÍ ===</f>
         <v/>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Žádný dokument neobsahuje preferenční větu (prohlášení o preferenčním původu).</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Původ zboží: USA. EU nemá s USA preferenční obchodní dohodu → preferenci nelze uplatnit a věta se ani nevyžaduje.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Platí smluvní sazby třetí země (viz výše). DPH 21 %.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="12">
-        <f>== ⚠️ NESROVNALOSTI K VYJASNĚNÍ ===</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>1) POČET KUSŮ: faktura 1 015 ks vs. HBL/MBL/D/O 1 032 ks (SLAC). Rozdíl 17 ks – vyjasnit se shipperem/forwarderem.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>2) HMOTNOSTI: faktura Net 44 000 lbs = 19 958,06 kg; sloupec Gross (KGS) 19 958 kg je jen přepočet lbs→kg (není to skutečná GW).</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   B/L gross 19 935 kg &lt; „net“ 19 958 kg → fyzicky nemožné. Skutečná NET hmotnost chybí – vyžádat od shippera.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Pro JSD zatím: GW 19 935 kg (dle B/L), rozdělena proporcionálně dle NET; NW nutno doložit.</t>
-        </is>
-      </c>
-    </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>3) INCOTERM: na faktuře není uveden; B/L „Freight Prepaid“. Ocean freight 3 700 USD hradí shipper → pro celní hodnotu</t>
+          <t>Žádný dokument neobsahuje preferenční větu (prohlášení o preferenčním původu).</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">   ověřit dodací podmínku (při CFR/CIF je přeprava již v ceně; při FOB/EXW nutno přičíst přepravu k celní hodnotě).</t>
+          <t>Původ zboží: USA. EU nemá s USA preferenční obchodní dohodu → preferenci nelze uplatnit a věta se ani nevyžaduje.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr"/>
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Platí smluvní sazby třetí země (viz výše). DPH 21 %.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="12">
+      <c r="A45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="12">
+        <f>== ⚠️ NESROVNALOSTI ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>1) POČET KUSŮ (TRVÁ): faktura 1 015 ks vs. HBL/MBL/D/O 1 032 ks (SLAC). Rozdíl 17 ks – vyjasnit se shipperem/forwarderem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2) HMOTNOSTI (VYŘEŠENO 17.7.2026): revidovaný CI/PL v2 uvádí NET 19 123 kg / GROSS 19 935 kg, souhlasí s B/L.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="12">
         <f>== CBAM / ANTIDUMPING ===</f>
         <v/>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
+    <row r="51">
+      <c r="A51" t="inlineStr">
         <is>
           <t>CBAM: nevztahuje se (kosmetické přípravky, mýdlo).</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
+    <row r="52">
+      <c r="A52" t="inlineStr">
         <is>
           <t>Antidumping: nevztahuje se (kap. 33/34, původ USA).</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="12">
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="12">
         <f>== SLEVA ===</f>
         <v/>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Žádná obchodní sleva na faktuře – celní hodnota bez úprav: 23 800,00 USD.</t>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Žádná obchodní sleva na faktuře – celní hodnota bez úprav: 23 800,00 USD + přeprava (viz Celní hodnota).</t>
         </is>
       </c>
     </row>

</xml_diff>